<commit_message>
Initial commit of Sales Installations Dashboard
</commit_message>
<xml_diff>
--- a/Access Master.xlsx
+++ b/Access Master.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harshal Thakkar\Dashboard\Sales &amp; Installation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harshal Thakkar\Dashboard\Sales &amp; Installation\sales-dashboard-rbac\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -41,9 +41,6 @@
     <t>Region/City</t>
   </si>
   <si>
-    <t>TP001</t>
-  </si>
-  <si>
     <t>manager1</t>
   </si>
   <si>
@@ -56,45 +53,30 @@
     <t>ALL</t>
   </si>
   <si>
-    <t>SM001</t>
-  </si>
-  <si>
     <t>manager2</t>
   </si>
   <si>
     <t>SMA_9999</t>
   </si>
   <si>
-    <t>HT001</t>
-  </si>
-  <si>
     <t>manager3</t>
   </si>
   <si>
     <t>H@rt2677</t>
   </si>
   <si>
-    <t>SN001</t>
-  </si>
-  <si>
     <t>manager4</t>
   </si>
   <si>
     <t>SNA_9978</t>
   </si>
   <si>
-    <t>GP001</t>
-  </si>
-  <si>
     <t>manager5</t>
   </si>
   <si>
     <t>GPA_5689</t>
   </si>
   <si>
-    <t>RB001</t>
-  </si>
-  <si>
     <t>lead1</t>
   </si>
   <si>
@@ -107,9 +89,6 @@
     <t>VADODARA,AHMEDABAD</t>
   </si>
   <si>
-    <t>SM002</t>
-  </si>
-  <si>
     <t>lead2</t>
   </si>
   <si>
@@ -119,9 +98,6 @@
     <t>PUNE,MUMBAI,CHENNAI,NAGPUR,BANGALORE,VISHAKAPATNAM,HYDERABAD,KAKINADA,VIJAYAWADA,AURANGABAD,NASHIK</t>
   </si>
   <si>
-    <t>AA001</t>
-  </si>
-  <si>
     <t>lead3</t>
   </si>
   <si>
@@ -129,6 +105,30 @@
   </si>
   <si>
     <t>RAJKOT</t>
+  </si>
+  <si>
+    <t>Tarpan Patel</t>
+  </si>
+  <si>
+    <t>Sameer Mahapatra</t>
+  </si>
+  <si>
+    <t>Harshal Thakkar</t>
+  </si>
+  <si>
+    <t>Sunish Nair</t>
+  </si>
+  <si>
+    <t>Gaurang Patel</t>
+  </si>
+  <si>
+    <t>Rajiv Bhatiya</t>
+  </si>
+  <si>
+    <t>Srinivas Mallavelli</t>
+  </si>
+  <si>
+    <t>Animesh Agarwal</t>
   </si>
 </sst>
 </file>
@@ -448,6 +448,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -468,138 +471,138 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
       <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
         <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
         <v>8</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
         <v>8</v>
-      </c>
-      <c r="E5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
         <v>8</v>
-      </c>
-      <c r="E6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>